<commit_message>
Add flat ECG CSV folder
</commit_message>
<xml_diff>
--- a/data/participant-datasets-by-catalog/participant_data_collection_catalog.xlsx
+++ b/data/participant-datasets-by-catalog/participant_data_collection_catalog.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Participant Overview" sheetId="1" r:id="Rf77eda2a51ea4015"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Codebook" sheetId="2" r:id="Rd6b6e5ab32cb49da"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Participant Overview" sheetId="1" r:id="Re0e6b3b3e11d4493"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Codebook" sheetId="2" r:id="Rbc09d8da8b0f4062"/>
   </x:sheets>
 </x:workbook>
 </file>

</xml_diff>

<commit_message>
Add P01 dynamic condition from headset sync
</commit_message>
<xml_diff>
--- a/data/participant-datasets-by-catalog/participant_data_collection_catalog.xlsx
+++ b/data/participant-datasets-by-catalog/participant_data_collection_catalog.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Participant Overview" sheetId="1" r:id="Re0e6b3b3e11d4493"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Codebook" sheetId="2" r:id="Rbc09d8da8b0f4062"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Participant Overview" sheetId="1" r:id="R18ee5569e3374e51"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Codebook" sheetId="2" r:id="R270938304e864ec0"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -339,13 +339,25 @@
       <x:c r="A2" s="8" t="str">
         <x:v>P01</x:v>
       </x:c>
-      <x:c r="B2" s="9" t="str"/>
-      <x:c r="C2" s="4" t="str"/>
-      <x:c r="D2" s="4" t="str"/>
-      <x:c r="E2" s="4" t="str"/>
+      <x:c r="B2" s="9" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="C2" s="4" t="str">
+        <x:v>female</x:v>
+      </x:c>
+      <x:c r="D2" s="4" t="str">
+        <x:v>right</x:v>
+      </x:c>
+      <x:c r="E2" s="4" t="str">
+        <x:v>yes</x:v>
+      </x:c>
       <x:c r="F2" s="4" t="str"/>
-      <x:c r="G2" s="4" t="str"/>
-      <x:c r="H2" s="4" t="str"/>
+      <x:c r="G2" s="4" t="str">
+        <x:v>Hand</x:v>
+      </x:c>
+      <x:c r="H2" s="4" t="str">
+        <x:v>incomplete</x:v>
+      </x:c>
       <x:c r="I2" s="4" t="str"/>
     </x:row>
     <x:row r="3" ht="26" customHeight="1">

</xml_diff>

<commit_message>
Add P14 dynamic condition from headset sync
</commit_message>
<xml_diff>
--- a/data/participant-datasets-by-catalog/participant_data_collection_catalog.xlsx
+++ b/data/participant-datasets-by-catalog/participant_data_collection_catalog.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Participant Overview" sheetId="1" r:id="R18ee5569e3374e51"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Codebook" sheetId="2" r:id="R270938304e864ec0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Participant Overview" sheetId="1" r:id="Rb72a87c3a517454a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Codebook" sheetId="2" r:id="Rff9ab617a89e4386"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -625,7 +625,9 @@
       <x:c r="D15" s="4" t="str">
         <x:v>left</x:v>
       </x:c>
-      <x:c r="E15" s="4" t="str"/>
+      <x:c r="E15" s="4" t="str">
+        <x:v>yes</x:v>
+      </x:c>
       <x:c r="F15" s="4" t="str">
         <x:v>yes</x:v>
       </x:c>
@@ -633,7 +635,7 @@
         <x:v>Env</x:v>
       </x:c>
       <x:c r="H15" s="4" t="str">
-        <x:v>incomplete</x:v>
+        <x:v>complete</x:v>
       </x:c>
       <x:c r="I15" s="4" t="str"/>
     </x:row>

</xml_diff>

<commit_message>
Refresh public data package
</commit_message>
<xml_diff>
--- a/data/participant-datasets-by-catalog/participant_data_collection_catalog.xlsx
+++ b/data/participant-datasets-by-catalog/participant_data_collection_catalog.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Participant Overview" sheetId="1" r:id="Rea76e0c6507048a1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Codebook" sheetId="2" r:id="Rda4ba175dd3e476e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Participant Overview" sheetId="1" r:id="R76c3cf6d3a8b4f47"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Codebook" sheetId="2" r:id="R44c82fc5edf94cb4"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -376,12 +376,14 @@
       <x:c r="E3" s="4" t="str">
         <x:v>yes</x:v>
       </x:c>
-      <x:c r="F3" s="4" t="str"/>
+      <x:c r="F3" s="4" t="str">
+        <x:v>yes</x:v>
+      </x:c>
       <x:c r="G3" s="4" t="str">
         <x:v>Hand</x:v>
       </x:c>
       <x:c r="H3" s="4" t="str">
-        <x:v>incomplete</x:v>
+        <x:v>complete</x:v>
       </x:c>
       <x:c r="I3" s="4" t="str"/>
     </x:row>
@@ -577,12 +579,14 @@
       <x:c r="E12" s="4" t="str">
         <x:v>yes</x:v>
       </x:c>
-      <x:c r="F12" s="4" t="str"/>
+      <x:c r="F12" s="4" t="str">
+        <x:v>yes</x:v>
+      </x:c>
       <x:c r="G12" s="4" t="str">
         <x:v>Hand</x:v>
       </x:c>
       <x:c r="H12" s="4" t="str">
-        <x:v>incomplete</x:v>
+        <x:v>complete</x:v>
       </x:c>
       <x:c r="I12" s="4" t="str"/>
     </x:row>

</xml_diff>